<commit_message>
Render Box 8/9 (EU supplies/acquisitions) transactions in working paper
_sheet_txn_by_box never rendered Box 8/Box 9 sub-sections, even though
TxnByBoxParser correctly parses them from the Xero export -- their
transaction detail was silently dropped from the "1B. Transactions by
VAT Box" sheet (confirmed against the real demo file, which has a real
Box 8 transaction). Box 1/4/6/7's existing hard-coded sub-label lookups
are unchanged; Box 8/9 use a small dynamic helper that renders whatever
sub-labels TxnByBoxParser actually parsed, rather than guessing an
unconfirmed Box 9 sub-label.

Regenerated scenario workbooks now genuinely include the new Box 8/9
rows where the underlying VAT Return has Box 8/9 data.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017XGczxhJJniAZqSzbUxS1o
</commit_message>
<xml_diff>
--- a/test_scenarios/accrual/VAT_Working_Papers_Demo_Company_UK_-_accrual_28_Feb_2026.xlsx
+++ b/test_scenarios/accrual/VAT_Working_Papers_Demo_Company_UK_-_accrual_28_Feb_2026.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="0. File Register" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1A. VAT Return" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1B. Txns by VAT Box" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2A. VAT Control" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2B. Bank Rec" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2C. Box 6 Rec" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3A. Aged Payables" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3B. Aged Receivables" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3C. Trial Balance" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4A. Top 10 Box 4" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VAT Checklist" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="0. File Register" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="1A. VAT Return" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="1B. Txns by VAT Box" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="2A. VAT Control" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="2B. Bank Rec" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="2C. Box 6 Rec" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="3A. Aged Payables" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="3B. Aged Receivables" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="3C. Trial Balance" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="4A. Top 10 Box 4" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="VAT Checklist" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -618,7 +618,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Generated:        25 Jun 2026 06:34</t>
+          <t>Generated:        20 Sep 2026 07:05</t>
         </is>
       </c>
     </row>
@@ -1821,7 +1821,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F135"/>
+  <dimension ref="A1:F144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4897,8 +4897,105 @@
         <v>103.43</v>
       </c>
     </row>
+    <row r="138">
+      <c r="A138" s="14" t="inlineStr">
+        <is>
+          <t>Box 8</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>EU supplies (NI)</t>
+        </is>
+      </c>
+      <c r="F138" s="11" t="n">
+        <v>1995</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="4" t="inlineStr">
+        <is>
+          <t>Zero Rated EC Goods Income</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="4" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B140" s="4" t="inlineStr">
+        <is>
+          <t>Account</t>
+        </is>
+      </c>
+      <c r="C140" s="4" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="D140" s="4" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+      <c r="E140" s="5" t="inlineStr">
+        <is>
+          <t>VAT (£)</t>
+        </is>
+      </c>
+      <c r="F140" s="5" t="inlineStr">
+        <is>
+          <t>Net (£)</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="3" t="inlineStr">
+        <is>
+          <t>23/02/2026</t>
+        </is>
+      </c>
+      <c r="B141" s="3" t="inlineStr">
+        <is>
+          <t>Sales(200)</t>
+        </is>
+      </c>
+      <c r="C141" s="3" t="inlineStr">
+        <is>
+          <t>INV-0042</t>
+        </is>
+      </c>
+      <c r="D141" s="3" t="inlineStr">
+        <is>
+          <t>Port &amp; Philip Freight - Fish out of Water: Finding Your Brand</t>
+        </is>
+      </c>
+      <c r="E141" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F141" s="15" t="n">
+        <v>1995</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="16" t="inlineStr">
+        <is>
+          <t>Box 9</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>EU acquisitions (NI)</t>
+        </is>
+      </c>
+      <c r="F144" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="16">
     <mergeCell ref="A73:F73"/>
     <mergeCell ref="A11:F11"/>
     <mergeCell ref="A101:B101"/>
@@ -4910,7 +5007,10 @@
     <mergeCell ref="A132:F132"/>
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="A126:F126"/>
+    <mergeCell ref="A138:B138"/>
+    <mergeCell ref="A139:F139"/>
     <mergeCell ref="A96:F96"/>
+    <mergeCell ref="A144:B144"/>
     <mergeCell ref="A35:B35"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>